<commit_message>
BOQ Bill 4: cupboard ironmongery per leaf + flush bolts per double door (Tom 19.10)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/ES26-081 BOQ Package.xlsx
+++ b/downloads/ES26-081 BOQ Package.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Bill 3 Internal Linings'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Bill 3 Internal Linings'!$A$1:$L$43</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Bill 4 Doors'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'Bill 4 Doors'!$A$1:$L$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Bill 4 Doors'!$A$1:$L$39</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Bill 5 Joinery'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Bill 5 Joinery'!$A$1:$L$49</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Bill 6 Partitions'!$6:$6</definedName>
@@ -1396,15 +1396,15 @@
         </is>
       </c>
       <c r="D21" s="11">
-        <f>'Bill 4 Doors'!I37</f>
+        <f>'Bill 4 Doors'!I38</f>
         <v/>
       </c>
       <c r="E21" s="11">
-        <f>'Bill 4 Doors'!J37</f>
+        <f>'Bill 4 Doors'!J38</f>
         <v/>
       </c>
       <c r="F21" s="11">
-        <f>'Bill 4 Doors'!K37</f>
+        <f>'Bill 4 Doors'!K38</f>
         <v/>
       </c>
     </row>
@@ -5564,15 +5564,15 @@
         </is>
       </c>
       <c r="D19" s="11">
-        <f>'Bill 4 Doors'!I34</f>
+        <f>'Bill 4 Doors'!I35</f>
         <v/>
       </c>
       <c r="E19" s="11">
-        <f>'Bill 4 Doors'!J34</f>
+        <f>'Bill 4 Doors'!J35</f>
         <v/>
       </c>
       <c r="F19" s="11">
-        <f>'Bill 4 Doors'!K34</f>
+        <f>'Bill 4 Doors'!K35</f>
         <v/>
       </c>
     </row>
@@ -5591,15 +5591,15 @@
         </is>
       </c>
       <c r="D20" s="11">
-        <f>'Bill 4 Doors'!I35</f>
+        <f>'Bill 4 Doors'!I36</f>
         <v/>
       </c>
       <c r="E20" s="11">
-        <f>'Bill 4 Doors'!J35</f>
+        <f>'Bill 4 Doors'!J36</f>
         <v/>
       </c>
       <c r="F20" s="11">
-        <f>'Bill 4 Doors'!K35</f>
+        <f>'Bill 4 Doors'!K36</f>
         <v/>
       </c>
     </row>
@@ -5618,15 +5618,15 @@
         </is>
       </c>
       <c r="D21" s="11">
-        <f>'Bill 4 Doors'!I36</f>
+        <f>'Bill 4 Doors'!I37</f>
         <v/>
       </c>
       <c r="E21" s="11">
-        <f>'Bill 4 Doors'!J36</f>
+        <f>'Bill 4 Doors'!J37</f>
         <v/>
       </c>
       <c r="F21" s="11">
-        <f>'Bill 4 Doors'!K36</f>
+        <f>'Bill 4 Doors'!K37</f>
         <v/>
       </c>
     </row>
@@ -5637,15 +5637,15 @@
         </is>
       </c>
       <c r="D22" s="13">
-        <f>'Bill 4 Doors'!I37</f>
+        <f>'Bill 4 Doors'!I38</f>
         <v/>
       </c>
       <c r="E22" s="13">
-        <f>'Bill 4 Doors'!J37</f>
+        <f>'Bill 4 Doors'!J38</f>
         <v/>
       </c>
       <c r="F22" s="13">
-        <f>'Bill 4 Doors'!K37</f>
+        <f>'Bill 4 Doors'!K38</f>
         <v/>
       </c>
     </row>
@@ -9155,7 +9155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9985,19 +9985,19 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Cupboard sets: catch and pull (flush bolt to pairs)</t>
+          <t>Cupboard sets per leaf: catch and pull</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>pr</t>
+          <t>set</t>
         </is>
       </c>
       <c r="D25" s="35" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E25" s="35" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F25" s="35">
         <f>D25+E25</f>
@@ -10019,11 +10019,11 @@
       </c>
       <c r="L25" s="38" t="inlineStr">
         <is>
-          <t>Doorsets; 7 leaves</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="26" customHeight="1">
+          <t>Per leaf; 5 doorsets</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
           <t>4B.5</t>
@@ -10031,7 +10031,7 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>FD30S sets: rated hinges, overhead closer, intumescent and smoke seals, signage</t>
+          <t>Flush bolts to cupboard double doors (fixed leaf)</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
@@ -10040,10 +10040,10 @@
         </is>
       </c>
       <c r="D26" s="35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" s="35">
         <f>D26+E26</f>
@@ -10065,72 +10065,72 @@
       </c>
       <c r="L26" s="38" t="inlineStr">
         <is>
+          <t>One per double door</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>4B.6</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>FD30S sets: rated hinges, overhead closer, intumescent and smoke seals, signage</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="D27" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="35">
+        <f>D27+E27</f>
+        <v/>
+      </c>
+      <c r="G27" s="36" t="n"/>
+      <c r="H27" s="36" t="n"/>
+      <c r="I27" s="11">
+        <f>F27*G27</f>
+        <v/>
+      </c>
+      <c r="J27" s="11">
+        <f>F27*H27</f>
+        <v/>
+      </c>
+      <c r="K27" s="37">
+        <f>I27+J27</f>
+        <v/>
+      </c>
+      <c r="L27" s="38" t="inlineStr">
+        <is>
           <t>Under-stair store - precaution, confirm with Building Control</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="30" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
         <is>
           <t>4C  External doorsets (for information - supply by others)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>4C.1</t>
         </is>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>GF flat entrance door (XD02), 1040 x 2100 structural opening, Front elevation; PAS 24 / SBD external doorset</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>nr</t>
-        </is>
-      </c>
-      <c r="D28" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="35">
-        <f>D28+E28</f>
-        <v/>
-      </c>
-      <c r="G28" s="36" t="n"/>
-      <c r="H28" s="36" t="n"/>
-      <c r="I28" s="11">
-        <f>F28*G28</f>
-        <v/>
-      </c>
-      <c r="J28" s="11">
-        <f>F28*H28</f>
-        <v/>
-      </c>
-      <c r="K28" s="37">
-        <f>I28+J28</f>
-        <v/>
-      </c>
-      <c r="L28" s="38" t="inlineStr">
-        <is>
-          <t>Window / door package - coordination only</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="39" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>4C.2</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>FF flat entrance door, stair lobby (WG01), 1040 x 2100 structural opening, Stair-lobby front elevation; PAS 24 / SBD external doorset</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -10168,15 +10168,15 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="26" customHeight="1">
+    <row r="30" ht="39" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>4C.3</t>
+          <t>4C.2</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>GF rear door, living/kitchen, 1040 x 2100 structural opening, Rear elevation; PAS 24 / SBD external doorset</t>
+          <t>FF flat entrance door, stair lobby (WG01), 1040 x 2100 structural opening, Stair-lobby front elevation; PAS 24 / SBD external doorset</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -10214,89 +10214,105 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="23" t="inlineStr">
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>4C.3</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>GF rear door, living/kitchen, 1040 x 2100 structural opening, Rear elevation; PAS 24 / SBD external doorset</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
+      <c r="D31" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="35">
+        <f>D31+E31</f>
+        <v/>
+      </c>
+      <c r="G31" s="36" t="n"/>
+      <c r="H31" s="36" t="n"/>
+      <c r="I31" s="11">
+        <f>F31*G31</f>
+        <v/>
+      </c>
+      <c r="J31" s="11">
+        <f>F31*H31</f>
+        <v/>
+      </c>
+      <c r="K31" s="37">
+        <f>I31+J31</f>
+        <v/>
+      </c>
+      <c r="L31" s="38" t="inlineStr">
+        <is>
+          <t>Window / door package - coordination only</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>PACKAGE SUMMARY  -  Bill 4  Internal Doors &amp; Ironmongery  (package JOI; amounts by others, excl. VAT)</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="9" t="inlineStr">
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C33" s="26" t="n"/>
-      <c r="D33" s="26" t="n"/>
-      <c r="E33" s="26" t="n"/>
-      <c r="F33" s="26" t="n"/>
-      <c r="G33" s="26" t="n"/>
-      <c r="H33" s="27" t="n"/>
-      <c r="I33" s="9" t="inlineStr">
+      <c r="C34" s="26" t="n"/>
+      <c r="D34" s="26" t="n"/>
+      <c r="E34" s="26" t="n"/>
+      <c r="F34" s="26" t="n"/>
+      <c r="G34" s="26" t="n"/>
+      <c r="H34" s="27" t="n"/>
+      <c r="I34" s="9" t="inlineStr">
         <is>
           <t>Supply
 £</t>
         </is>
       </c>
-      <c r="J33" s="9" t="inlineStr">
+      <c r="J34" s="9" t="inlineStr">
         <is>
           <t>Install
 £</t>
         </is>
       </c>
-      <c r="K33" s="9" t="inlineStr">
+      <c r="K34" s="9" t="inlineStr">
         <is>
           <t>Total
 £</t>
         </is>
       </c>
-      <c r="L33" s="9" t="inlineStr"/>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="39" t="inlineStr">
-        <is>
-          <t>4A</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>Internal doorsets (NRM2 24 / package JOI)</t>
-        </is>
-      </c>
-      <c r="C34" s="16" t="n"/>
-      <c r="D34" s="16" t="n"/>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="16" t="n"/>
-      <c r="G34" s="16" t="n"/>
-      <c r="H34" s="16" t="n"/>
-      <c r="I34" s="11">
-        <f>SUM(I8:I20)</f>
-        <v/>
-      </c>
-      <c r="J34" s="11">
-        <f>SUM(J8:J20)</f>
-        <v/>
-      </c>
-      <c r="K34" s="37">
-        <f>SUM(K8:K20)</f>
-        <v/>
-      </c>
+      <c r="L34" s="9" t="inlineStr"/>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="39" t="inlineStr">
         <is>
-          <t>4B</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Ironmongery (NRM2 24 / package JOI)</t>
+          <t>Internal doorsets (NRM2 24 / package JOI)</t>
         </is>
       </c>
       <c r="C35" s="16" t="n"/>
@@ -10306,27 +10322,27 @@
       <c r="G35" s="16" t="n"/>
       <c r="H35" s="16" t="n"/>
       <c r="I35" s="11">
-        <f>SUM(I22:I26)</f>
+        <f>SUM(I8:I20)</f>
         <v/>
       </c>
       <c r="J35" s="11">
-        <f>SUM(J22:J26)</f>
+        <f>SUM(J8:J20)</f>
         <v/>
       </c>
       <c r="K35" s="37">
-        <f>SUM(K22:K26)</f>
+        <f>SUM(K8:K20)</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="39" t="inlineStr">
         <is>
-          <t>4C</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>External doorsets (for information - supply by others)</t>
+          <t>Ironmongery (NRM2 24 / package JOI)</t>
         </is>
       </c>
       <c r="C36" s="16" t="n"/>
@@ -10336,39 +10352,69 @@
       <c r="G36" s="16" t="n"/>
       <c r="H36" s="16" t="n"/>
       <c r="I36" s="11">
-        <f>SUM(I28:I30)</f>
+        <f>SUM(I22:I27)</f>
         <v/>
       </c>
       <c r="J36" s="11">
-        <f>SUM(J28:J30)</f>
+        <f>SUM(J22:J27)</f>
         <v/>
       </c>
       <c r="K36" s="37">
-        <f>SUM(K28:K30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="40" t="inlineStr">
+        <f>SUM(K22:K27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="39" t="inlineStr">
+        <is>
+          <t>4C</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>External doorsets (for information - supply by others)</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="n"/>
+      <c r="D37" s="16" t="n"/>
+      <c r="E37" s="16" t="n"/>
+      <c r="F37" s="16" t="n"/>
+      <c r="G37" s="16" t="n"/>
+      <c r="H37" s="16" t="n"/>
+      <c r="I37" s="11">
+        <f>SUM(I29:I31)</f>
+        <v/>
+      </c>
+      <c r="J37" s="11">
+        <f>SUM(J29:J31)</f>
+        <v/>
+      </c>
+      <c r="K37" s="37">
+        <f>SUM(K29:K31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="40" t="inlineStr">
         <is>
           <t>PACKAGE TOTAL - Bill 4, carried to the Cover overview</t>
         </is>
       </c>
-      <c r="I37" s="13">
-        <f>SUM(I34:I36)</f>
-        <v/>
-      </c>
-      <c r="J37" s="13">
-        <f>SUM(J34:J36)</f>
-        <v/>
-      </c>
-      <c r="K37" s="13">
-        <f>SUM(K34:K36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="21" t="inlineStr">
+      <c r="I38" s="13">
+        <f>SUM(I35:I37)</f>
+        <v/>
+      </c>
+      <c r="J38" s="13">
+        <f>SUM(J35:J37)</f>
+        <v/>
+      </c>
+      <c r="K38" s="13">
+        <f>SUM(K35:K37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="21" t="inlineStr">
         <is>
           <t>Pale-yellow cells are the only inputs (Supply rate, Install rate). Amounts, subtotals and totals are formulas; the sheet is protected without a password (Review &gt; Unprotect Sheet). Amounts exclude VAT and are NOT part of the Nudura ICF price.</t>
         </is>
@@ -10378,14 +10424,14 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="14">
     <mergeCell ref="B36:H36"/>
-    <mergeCell ref="A38:L38"/>
     <mergeCell ref="A21:L21"/>
     <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A39:L39"/>
+    <mergeCell ref="A33:L33"/>
     <mergeCell ref="B35:H35"/>
-    <mergeCell ref="A32:L32"/>
-    <mergeCell ref="B33:H33"/>
-    <mergeCell ref="A27:L27"/>
-    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="B37:H37"/>
     <mergeCell ref="C2:L2"/>
     <mergeCell ref="B34:H34"/>
     <mergeCell ref="C1:L1"/>

</xml_diff>